<commit_message>
EPBDS-16819 Fix a named constructor argument reading the field of the new object, which made new Customer(name = name) leave the name null
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.test/test-resources/functionality/EPBDS-7063.xlsx
+++ b/DEV/org.openl.rules.test/test-resources/functionality/EPBDS-7063.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="192">
   <si>
     <t>String</t>
   </si>
@@ -175,7 +175,7 @@
     <t>type2type3num3</t>
   </si>
   <si>
-    <t>//Test spr3 spr3Test</t>
+    <t>Test spr3 spr3Test</t>
   </si>
   <si>
     <t xml:space="preserve">// Constructir fo the datatype with inheritance </t>
@@ -1609,11 +1609,9 @@
       <c r="D41" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="E41" s="12" t="s">
-        <v>11</v>
-      </c>
+      <c r="E41" s="12"/>
       <c r="F41" s="12">
-        <v>2</v>
+        <v>111</v>
       </c>
       <c r="G41" s="12">
         <v>222</v>

</xml_diff>